<commit_message>
Updated Metrics Results and Started PowerPoint
</commit_message>
<xml_diff>
--- a/Proyecto/entrenamiento/figures/metrics_comparison/Evaluacion_Avanzada.xlsx
+++ b/Proyecto/entrenamiento/figures/metrics_comparison/Evaluacion_Avanzada.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danil\OneDrive\Escritorio\Universidad\Cuarto\TFG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D25EB8E5-FF3E-4734-99AA-C5AECD3149C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7AC3058-7E7C-4977-8E1E-C451A8B61083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{FFE60E07-585A-457C-B0E2-6C20AE62698F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{FFE60E07-585A-457C-B0E2-6C20AE62698F}"/>
   </bookViews>
   <sheets>
     <sheet name="ShiftedMAPE" sheetId="1" r:id="rId1"/>
@@ -189,13 +189,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -533,13 +533,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6D9E335-44A9-45DF-AB8C-72B4E23D68AE}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.36328125" customWidth="1"/>
-    <col min="2" max="10" width="18.81640625" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" customWidth="1"/>
+    <col min="2" max="10" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4"/>
       <c r="B1" s="7" t="s">
         <v>10</v>
@@ -557,7 +557,7 @@
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
     </row>
-    <row r="2" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -589,7 +589,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -621,7 +621,7 @@
         <v>0.54455500000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
@@ -653,7 +653,7 @@
         <v>0.88461900000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -685,7 +685,7 @@
         <v>0.88299899999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
@@ -717,7 +717,7 @@
         <v>0.86690299999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
@@ -749,7 +749,7 @@
         <v>0.83809299999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>9</v>
       </c>
@@ -781,7 +781,7 @@
         <v>0.88229999999999997</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
@@ -813,7 +813,7 @@
         <v>0.86145400000000005</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:10" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
@@ -966,31 +966,31 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DF62460-7224-49F9-B7E7-FCC9BA4C52DE}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.6328125" customWidth="1"/>
-    <col min="2" max="10" width="16.6328125" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" customWidth="1"/>
+    <col min="2" max="10" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6" t="s">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6" t="s">
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-    </row>
-    <row r="2" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+    </row>
+    <row r="2" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1054,7 +1054,7 @@
         <v>0.54455529999999996</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -1086,7 +1086,7 @@
         <v>0.88461909999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>0.88299899999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -1150,7 +1150,7 @@
         <v>0.86690310000000004</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1182,7 +1182,7 @@
         <v>0.83809350000000005</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="29.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:10" ht="29.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -1214,7 +1214,7 @@
         <v>0.88230039999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="29.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:10" ht="29.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -1224,7 +1224,7 @@
       <c r="C9" s="2">
         <v>1.725E-3</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="6">
         <v>0.97456200000000004</v>
       </c>
       <c r="E9" s="2">
@@ -1246,7 +1246,7 @@
         <v>0.86145400000000005</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="29.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:10" ht="29.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
@@ -1285,6 +1285,30 @@
     <mergeCell ref="H1:J1"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B9">
+    <cfRule type="colorScale" priority="36">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B10">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
     <cfRule type="colorScale" priority="27">
       <colorScale>
         <cfvo type="min"/>
@@ -1296,8 +1320,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B10">
-    <cfRule type="colorScale" priority="18">
+  <conditionalFormatting sqref="C3:C8 C10">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1309,6 +1333,18 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:C8">
+    <cfRule type="colorScale" priority="35">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10">
     <cfRule type="colorScale" priority="26">
       <colorScale>
         <cfvo type="min"/>
@@ -1320,19 +1356,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C10">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D3:D8 C9:D9">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D8 D10 C9:D9">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D10">
     <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
@@ -1344,195 +1392,15 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D10">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="E3:E9">
-    <cfRule type="colorScale" priority="25">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E10">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F9">
-    <cfRule type="colorScale" priority="24">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F10">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G9">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G10">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H9">
-    <cfRule type="colorScale" priority="23">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H10">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I9">
-    <cfRule type="colorScale" priority="22">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I10">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J3:J9">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J10">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3:B10">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C8 C10">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D8 D10 C9:D9">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
+    <cfRule type="colorScale" priority="34">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -1548,6 +1416,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E10">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:F9">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F3:F10">
     <cfRule type="colorScale" priority="5">
       <colorScale>
@@ -1560,6 +1452,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F10">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3:G9">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G3:G10">
     <cfRule type="colorScale" priority="4">
       <colorScale>
@@ -1572,6 +1488,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G10">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H9">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H3:H10">
     <cfRule type="colorScale" priority="3">
       <colorScale>
@@ -1584,6 +1524,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H10">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:I9">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I3:I10">
     <cfRule type="colorScale" priority="2">
       <colorScale>
@@ -1596,6 +1560,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I10">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J9">
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J3:J10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -1605,6 +1593,42 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J10">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D10">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C10">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>

</xml_diff>